<commit_message>
Venere: allineamento completo dei documenti al regime ambulatorio + decisioni
- Deck v7 (seed = 1 ambulatorio pilota + 3 LOI blindate)
- DECISIONE, PIANO_OPERATIVO, PIANO_ESECUTIVO, Format_Playbook: banner + fix (ambulatorio, hub&spoke, Marcello maxillo-facciale/DS, DO Fase 2, capex)
- Lista_Target_Starter riscritta su centri estetici/ATECO 96.02.02
- Guida_Qualifica, Piano_90: barra ambulatorio
- Modello finanziario: capex ~350k/sede, seed pilota, MOIC/ambulatorio 3,97x
- README indice dossier; PDF rigenerati (memo, piano esecutivo, format, guida, lista)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QhepYozFjjk17WbLpFAXS3
</commit_message>
<xml_diff>
--- a/Venere_Modello_Finanziario.xlsx
+++ b/Venere_Modello_Finanziario.xlsx
@@ -21,12 +21,12 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="€#,##0;(€#,##0);-"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
-    <numFmt numFmtId="166" formatCode="0.0x"/>
+    <numFmt numFmtId="164" formatCode="0.0x"/>
+    <numFmt numFmtId="165" formatCode="€#,##0;(€#,##0);-"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="#,##0;(#,##0);-"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -84,6 +84,10 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000000CC"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -115,35 +119,50 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="10" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="10" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -527,7 +546,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Base case, numeri illustrativi da validare in DD. Il file RICALCOLA all'apertura in Excel o Google Sheets.</t>
+          <t>Base case regime AMBULATORIO, numeri illustrativi da validare in DD. Il file RICALCOLA all'apertura in Excel o Google Sheets.</t>
         </is>
       </c>
     </row>
@@ -542,10 +561,10 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>MOIC per centro convertito</t>
-        </is>
-      </c>
-      <c r="B5" s="6">
+          <t>MOIC per ambulatorio convertito</t>
+        </is>
+      </c>
+      <c r="B5" s="24">
         <f>Unit_Economics!B21</f>
         <v/>
       </c>
@@ -556,7 +575,7 @@
           <t>Capitale investito per centro</t>
         </is>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="25">
         <f>Unit_Economics!B11</f>
         <v/>
       </c>
@@ -567,7 +586,7 @@
           <t>EBITDA a regime per centro</t>
         </is>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="25">
         <f>Unit_Economics!B15</f>
         <v/>
       </c>
@@ -578,19 +597,19 @@
           <t>Seed — totale impieghi (vs €500k)</t>
         </is>
       </c>
-      <c r="B8" s="7">
-        <f>Seed_500k!B7</f>
+      <c r="B8" s="25">
+        <f>Seed_500k!B8</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Seed — (deficit) per convertire tutti e 3</t>
-        </is>
-      </c>
-      <c r="B9" s="7">
-        <f>Seed_500k!B11</f>
+          <t>Seed — residuo dopo il pilota (LOI + WC)</t>
+        </is>
+      </c>
+      <c r="B9" s="25">
+        <f>Seed_500k!B12</f>
         <v/>
       </c>
     </row>
@@ -600,7 +619,7 @@
           <t>EBITDA gruppo Anno 5</t>
         </is>
       </c>
-      <c r="B10" s="7">
+      <c r="B10" s="25">
         <f>Gruppo_Returns!F8</f>
         <v/>
       </c>
@@ -611,7 +630,7 @@
           <t>Enterprise Value all'exit (Anno 5)</t>
         </is>
       </c>
-      <c r="B11" s="7">
+      <c r="B11" s="25">
         <f>Gruppo_Returns!B12</f>
         <v/>
       </c>
@@ -622,7 +641,7 @@
           <t>MOIC investitore seed</t>
         </is>
       </c>
-      <c r="B12" s="6">
+      <c r="B12" s="24">
         <f>Gruppo_Returns!E16</f>
         <v/>
       </c>
@@ -633,7 +652,7 @@
           <t>Valore fondatori all'exit</t>
         </is>
       </c>
-      <c r="B13" s="7">
+      <c r="B13" s="25">
         <f>Gruppo_Returns!D19</f>
         <v/>
       </c>
@@ -682,7 +701,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Numeri illustrativi, base case. Da validare in DD. Fonti: annunci subito.it/idealista, benchmark medspa USA, deck Venere.</t>
+          <t>Numeri illustrativi, base case (regime AMBULATORIO). Da validare in DD. Fonti: annunci idealista/immobiliare, benchmark medspa USA, deck Venere v7.</t>
         </is>
       </c>
     </row>
@@ -702,8 +721,8 @@
           <t>Ricavi centro all'acquisto</t>
         </is>
       </c>
-      <c r="B5" s="9" t="n">
-        <v>450000</v>
+      <c r="B5" s="26" t="n">
+        <v>600000</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
@@ -712,7 +731,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>centro estetico target con footfall reale</t>
+          <t>centro estetico affermato con footfall reale</t>
         </is>
       </c>
     </row>
@@ -722,7 +741,7 @@
           <t>Margine EBITDA all'acquisto</t>
         </is>
       </c>
-      <c r="B6" s="10" t="n">
+      <c r="B6" s="27" t="n">
         <v>0.15</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -737,27 +756,27 @@
           <t>Prezzo d'acquisto (cessione attività)</t>
         </is>
       </c>
-      <c r="B7" s="9" t="n">
-        <v>150000</v>
+      <c r="B7" s="26" t="n">
+        <v>270000</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>range €50-300k; mid con clientela</t>
+          <t>circa 3x EBITDA normalizzato (con clientela)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>Capex di conversione medica</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="n">
-        <v>180000</v>
+          <t>Capex di conversione in ambulatorio</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="n">
+        <v>350000</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>autorizzazione, sale, sterilizzazione, device (range 150-300k)</t>
+          <t>AMBULATORIO: locali distinti, impianti, autorizzazione, sterilizzazione, device (range 250-450k)</t>
         </is>
       </c>
     </row>
@@ -767,8 +786,8 @@
           <t>Ricavi a regime (medicalizzato, 24m)</t>
         </is>
       </c>
-      <c r="B9" s="9" t="n">
-        <v>850000</v>
+      <c r="B9" s="26" t="n">
+        <v>1100000</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -777,7 +796,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>beauty + medicina estetica su base clienti</t>
+          <t>beauty + medicina estetica in ambulatorio, su base clienti</t>
         </is>
       </c>
     </row>
@@ -787,7 +806,7 @@
           <t>Margine EBITDA a regime</t>
         </is>
       </c>
-      <c r="B10" s="10" t="n">
+      <c r="B10" s="27" t="n">
         <v>0.28</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -802,7 +821,7 @@
           <t>Multiplo di uscita (EBITDA)</t>
         </is>
       </c>
-      <c r="B11" s="11" t="n">
+      <c r="B11" s="28" t="n">
         <v>8</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -817,7 +836,7 @@
           <t>Fattore di maturità dei ricavi (blended)</t>
         </is>
       </c>
-      <c r="B12" s="10" t="n">
+      <c r="B12" s="27" t="n">
         <v>0.8</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -842,12 +861,12 @@
           <t>Anno 1</t>
         </is>
       </c>
-      <c r="B15" s="12" t="n">
-        <v>2</v>
+      <c r="B15" s="29" t="n">
+        <v>1</v>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Anno 1 = seed (2 conversioni provate); da Anno 2 la scala</t>
+          <t>Anno 1 = seed (1 ambulatorio pilota); da Anno 2 la scala</t>
         </is>
       </c>
     </row>
@@ -857,8 +876,8 @@
           <t>Anno 2</t>
         </is>
       </c>
-      <c r="B16" s="12" t="n">
-        <v>6</v>
+      <c r="B16" s="29" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="17">
@@ -867,8 +886,8 @@
           <t>Anno 3</t>
         </is>
       </c>
-      <c r="B17" s="12" t="n">
-        <v>12</v>
+      <c r="B17" s="29" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="18">
@@ -877,8 +896,8 @@
           <t>Anno 4</t>
         </is>
       </c>
-      <c r="B18" s="12" t="n">
-        <v>20</v>
+      <c r="B18" s="29" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="19">
@@ -887,8 +906,8 @@
           <t>Anno 5</t>
         </is>
       </c>
-      <c r="B19" s="12" t="n">
-        <v>28</v>
+      <c r="B19" s="29" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="21">
@@ -907,7 +926,7 @@
           <t>Anno 1</t>
         </is>
       </c>
-      <c r="B22" s="9" t="n">
+      <c r="B22" s="30" t="n">
         <v>300000</v>
       </c>
     </row>
@@ -917,7 +936,7 @@
           <t>Anno 2</t>
         </is>
       </c>
-      <c r="B23" s="9" t="n">
+      <c r="B23" s="30" t="n">
         <v>600000</v>
       </c>
     </row>
@@ -927,7 +946,7 @@
           <t>Anno 3</t>
         </is>
       </c>
-      <c r="B24" s="9" t="n">
+      <c r="B24" s="30" t="n">
         <v>1000000</v>
       </c>
     </row>
@@ -937,7 +956,7 @@
           <t>Anno 4</t>
         </is>
       </c>
-      <c r="B25" s="9" t="n">
+      <c r="B25" s="30" t="n">
         <v>1400000</v>
       </c>
     </row>
@@ -947,7 +966,7 @@
           <t>Anno 5</t>
         </is>
       </c>
-      <c r="B26" s="9" t="n">
+      <c r="B26" s="30" t="n">
         <v>1800000</v>
       </c>
     </row>
@@ -967,12 +986,12 @@
           <t>Seed (l'ask di oggi)</t>
         </is>
       </c>
-      <c r="B29" s="9" t="n">
+      <c r="B29" s="30" t="n">
         <v>500000</v>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>provare il modello su 3 centri</t>
+          <t>provare 1 ambulatorio pilota + blindare 3 LOI</t>
         </is>
       </c>
     </row>
@@ -982,7 +1001,7 @@
           <t>Seed — post-money</t>
         </is>
       </c>
-      <c r="B30" s="9" t="n">
+      <c r="B30" s="30" t="n">
         <v>3500000</v>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -997,12 +1016,12 @@
           <t>Round di scala</t>
         </is>
       </c>
-      <c r="B31" s="9" t="n">
-        <v>3000000</v>
+      <c r="B31" s="26" t="n">
+        <v>4000000</v>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>a modello provato (range 2,5-4,5M)</t>
+          <t>a modello provato (range 3-5M); converte i 3 + cluster</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1031,7 @@
           <t>Round di scala — post-money</t>
         </is>
       </c>
-      <c r="B32" s="9" t="n">
+      <c r="B32" s="30" t="n">
         <v>15000000</v>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1027,7 +1046,7 @@
           <t>Pool ESOP (management, incl. COO)</t>
         </is>
       </c>
-      <c r="B33" s="10" t="n">
+      <c r="B33" s="27" t="n">
         <v>0.12</v>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1039,7 +1058,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>SEED — sotto-assunzioni (primi centri, scrappy)</t>
+          <t>SEED — sotto-assunzioni (1 ambulatorio pilota + pipeline LOI)</t>
         </is>
       </c>
       <c r="B35" s="4" t="n"/>
@@ -1049,60 +1068,60 @@
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>Prezzo per centro (seed, piccolo)</t>
-        </is>
-      </c>
-      <c r="B36" s="9" t="n">
-        <v>80000</v>
+          <t>Cash al closing centro pilota</t>
+        </is>
+      </c>
+      <c r="B36" s="26" t="n">
+        <v>175000</v>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>salon piccoli da annunci (50-100k)</t>
+          <t>circa 65% del prezzo (o pilota economico + rollover)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>Capex conversione (seed, leggera)</t>
-        </is>
-      </c>
-      <c r="B37" s="9" t="n">
-        <v>130000</v>
+          <t>Capex conversione ambulatorio pilota (lean)</t>
+        </is>
+      </c>
+      <c r="B37" s="26" t="n">
+        <v>295000</v>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>sede in affitto, Marcello DS condiviso</t>
+          <t>contenuto; il capex pieno ~350k arriva in Series A</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>N centri comprati col seed</t>
-        </is>
-      </c>
-      <c r="B38" s="12" t="n">
-        <v>3</v>
+          <t>N ambulatori convertiti nel seed</t>
+        </is>
+      </c>
+      <c r="B38" s="29" t="n">
+        <v>1</v>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>pipeline: 3 di 5 che vendono</t>
+          <t>il pilota; gli altri 2 in Series A</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>N conversioni nel seed</t>
-        </is>
-      </c>
-      <c r="B39" s="12" t="n">
-        <v>2</v>
+          <t>Acconti/opzioni su 2 LOI aggiuntive</t>
+        </is>
+      </c>
+      <c r="B39" s="29" t="n">
+        <v>20000</v>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>gli altri convertiti col round di scala</t>
+          <t>blindare la pipeline per la Series A</t>
         </is>
       </c>
     </row>
@@ -1129,7 +1148,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Unit economics — un centro estetico convertito</t>
+          <t>Unit economics — un centro estetico convertito in ambulatorio</t>
         </is>
       </c>
     </row>
@@ -1149,7 +1168,7 @@
           <t>Ricavi</t>
         </is>
       </c>
-      <c r="B4" s="7">
+      <c r="B4" s="25">
         <f>Assunzioni!B5</f>
         <v/>
       </c>
@@ -1160,7 +1179,7 @@
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="31">
         <f>Assunzioni!B5*Assunzioni!B6</f>
         <v/>
       </c>
@@ -1171,7 +1190,7 @@
           <t>Prezzo d'acquisto</t>
         </is>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="25">
         <f>Assunzioni!B7</f>
         <v/>
       </c>
@@ -1182,7 +1201,7 @@
           <t>Multiplo implicito d'acquisto</t>
         </is>
       </c>
-      <c r="B7" s="14">
+      <c r="B7" s="32">
         <f>B6/B5</f>
         <v/>
       </c>
@@ -1195,7 +1214,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Medicalizzazione</t>
+          <t>Conversione in ambulatorio</t>
         </is>
       </c>
       <c r="B9" s="4" t="n"/>
@@ -1205,10 +1224,10 @@
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>Capex di conversione</t>
-        </is>
-      </c>
-      <c r="B10" s="7">
+          <t>Capex di conversione in ambulatorio</t>
+        </is>
+      </c>
+      <c r="B10" s="25">
         <f>Assunzioni!B8</f>
         <v/>
       </c>
@@ -1219,7 +1238,7 @@
           <t>Capitale investito totale</t>
         </is>
       </c>
-      <c r="B11" s="15">
+      <c r="B11" s="33">
         <f>B6+B10</f>
         <v/>
       </c>
@@ -1227,7 +1246,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>A regime (24 mesi)</t>
+          <t>A regime (24 mesi, ambulatorio)</t>
         </is>
       </c>
       <c r="B13" s="4" t="n"/>
@@ -1240,7 +1259,7 @@
           <t>Ricavi a regime</t>
         </is>
       </c>
-      <c r="B14" s="7">
+      <c r="B14" s="25">
         <f>Assunzioni!B9</f>
         <v/>
       </c>
@@ -1251,7 +1270,7 @@
           <t>EBITDA a regime</t>
         </is>
       </c>
-      <c r="B15" s="15">
+      <c r="B15" s="33">
         <f>Assunzioni!B9*Assunzioni!B10</f>
         <v/>
       </c>
@@ -1262,7 +1281,7 @@
           <t>Uplift EBITDA vs acquisto</t>
         </is>
       </c>
-      <c r="B16" s="13">
+      <c r="B16" s="31">
         <f>B15-B5</f>
         <v/>
       </c>
@@ -1283,7 +1302,7 @@
           <t>Valore a regime (EBITDA x multiplo)</t>
         </is>
       </c>
-      <c r="B19" s="15">
+      <c r="B19" s="33">
         <f>B15*Assunzioni!B11</f>
         <v/>
       </c>
@@ -1294,7 +1313,7 @@
           <t>Valore creato (netto del capitale investito)</t>
         </is>
       </c>
-      <c r="B20" s="13">
+      <c r="B20" s="31">
         <f>B19-B11</f>
         <v/>
       </c>
@@ -1305,7 +1324,7 @@
           <t>MOIC per centro (valore / capitale investito)</t>
         </is>
       </c>
-      <c r="B21" s="16">
+      <c r="B21" s="34">
         <f>B19/B11</f>
         <v/>
       </c>
@@ -1313,7 +1332,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Doppio arbitraggio: compri a sconto (multiplo basso) + medicalizzi (EBITDA su, re-rating a multiplo medico).</t>
+          <t>Doppio arbitraggio: compri a sconto (multiplo basso) + converti in ambulatorio (EBITDA su, re-rating a multiplo medico). Capex piu' alto dello studio medico: e' la barra che fa da fossato.</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1359,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Seed €500k — use of funds (cosa compra davvero)</t>
+          <t>Seed €500k — use of funds (cosa compra davvero, regime ambulatorio)</t>
         </is>
       </c>
     </row>
@@ -1357,111 +1376,123 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>Acquisto centri (n x prezzo seed)</t>
-        </is>
-      </c>
-      <c r="B4" s="7">
-        <f>Assunzioni!B38*Assunzioni!B36</f>
+          <t>Cash al closing centro pilota</t>
+        </is>
+      </c>
+      <c r="B4" s="25">
+        <f>Assunzioni!B36</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>Conversioni nel seed (n x capex leggera)</t>
-        </is>
-      </c>
-      <c r="B5" s="7">
-        <f>Assunzioni!B39*Assunzioni!B37</f>
+          <t>Capex conversione ambulatorio (pilota, lean)</t>
+        </is>
+      </c>
+      <c r="B5" s="25">
+        <f>Assunzioni!B37</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>Working capital + costi centrali di partenza</t>
-        </is>
-      </c>
-      <c r="B6" s="13">
-        <f>B9-B4-B5</f>
-        <v/>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>residuo del seed dopo acquisti e conversioni</t>
-        </is>
-      </c>
+          <t>Acconti/opzioni su 2 LOI aggiuntive</t>
+        </is>
+      </c>
+      <c r="B6" s="31">
+        <f>Assunzioni!B39</f>
+        <v/>
+      </c>
+      <c r="D6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Totale impieghi</t>
-        </is>
-      </c>
-      <c r="B7" s="15">
-        <f>B4+B5+B6</f>
-        <v/>
+          <t>Working capital + costi centrali di partenza</t>
+        </is>
+      </c>
+      <c r="B7" s="33">
+        <f>B10-B4-B5-B6</f>
+        <v/>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>residuo del seed</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Fonti e verifica</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="n"/>
+          <t>Totale impieghi</t>
+        </is>
+      </c>
+      <c r="B8" s="4">
+        <f>B4+B5+B6+B7</f>
+        <v/>
+      </c>
       <c r="C8" s="4" t="n"/>
       <c r="D8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Seed disponibile</t>
-        </is>
-      </c>
-      <c r="B9" s="15">
-        <f>Assunzioni!B29</f>
-        <v/>
-      </c>
+          <t>Fonti e verifica</t>
+        </is>
+      </c>
+      <c r="B9" s="33" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>Copre 3 conversioni complete? (fabbisogno)</t>
-        </is>
-      </c>
-      <c r="B10" s="13">
-        <f>Assunzioni!B38*(Assunzioni!B36+Assunzioni!B37)</f>
-        <v/>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>acquisto + conversione di TUTTI e 3</t>
-        </is>
-      </c>
+          <t>Seed disponibile</t>
+        </is>
+      </c>
+      <c r="B10" s="31">
+        <f>Assunzioni!B29</f>
+        <v/>
+      </c>
+      <c r="D10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Surplus / (deficit) per le 3 conversioni</t>
-        </is>
-      </c>
-      <c r="B11" s="17">
-        <f>B9-B10</f>
+          <t>Fabbisogno 1 pilota completo (closing + capex)</t>
+        </is>
+      </c>
+      <c r="B11" s="35">
+        <f>B4+B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Residuo dopo il pilota (per LOI + WC)</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>B10-B11</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Lettura onesta: €500k compra 3 centri e ne converte 2 (Marcello DS condiviso). La 3a conversione</t>
-        </is>
+          <t>Fabbisogno per convertire PIENAMENTE i 3 (Series A)</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>3*(Assunzioni!B7*0.65+Assunzioni!B8)</f>
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>e il capex pieno arrivano col round di scala. Per 3 conversioni complete subito servono ~€650-750k.</t>
+          <t>Lettura onesta: €500k converte 1 ambulatorio PILOTA e blinda 3 LOI (margine sottile). La conversione piena dei 3 e' la Series A (~€1,6M). Per un pilota comodo servirebbero ~€600-700k.</t>
         </is>
       </c>
     </row>
@@ -1556,23 +1587,23 @@
           <t>Ricavi gruppo</t>
         </is>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="31">
         <f>B4*Assunzioni!B9*Assunzioni!B12</f>
         <v/>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="31">
         <f>C4*Assunzioni!B9*Assunzioni!B12</f>
         <v/>
       </c>
-      <c r="D5" s="13">
+      <c r="D5" s="31">
         <f>D4*Assunzioni!B9*Assunzioni!B12</f>
         <v/>
       </c>
-      <c r="E5" s="13">
+      <c r="E5" s="31">
         <f>E4*Assunzioni!B9*Assunzioni!B12</f>
         <v/>
       </c>
-      <c r="F5" s="13">
+      <c r="F5" s="31">
         <f>F4*Assunzioni!B9*Assunzioni!B12</f>
         <v/>
       </c>
@@ -1583,23 +1614,23 @@
           <t>EBITDA sedi</t>
         </is>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="31">
         <f>B5*Assunzioni!B10</f>
         <v/>
       </c>
-      <c r="C6" s="13">
+      <c r="C6" s="31">
         <f>C5*Assunzioni!B10</f>
         <v/>
       </c>
-      <c r="D6" s="13">
+      <c r="D6" s="31">
         <f>D5*Assunzioni!B10</f>
         <v/>
       </c>
-      <c r="E6" s="13">
+      <c r="E6" s="31">
         <f>E5*Assunzioni!B10</f>
         <v/>
       </c>
-      <c r="F6" s="13">
+      <c r="F6" s="31">
         <f>F5*Assunzioni!B10</f>
         <v/>
       </c>
@@ -1610,23 +1641,23 @@
           <t>Costo piattaforma centrale</t>
         </is>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="25">
         <f>-Assunzioni!B22</f>
         <v/>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="25">
         <f>-Assunzioni!B23</f>
         <v/>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="25">
         <f>-Assunzioni!B24</f>
         <v/>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="25">
         <f>-Assunzioni!B25</f>
         <v/>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="25">
         <f>-Assunzioni!B26</f>
         <v/>
       </c>
@@ -1637,23 +1668,23 @@
           <t>EBITDA gruppo</t>
         </is>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="33">
         <f>B6+B7</f>
         <v/>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="33">
         <f>C6+C7</f>
         <v/>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="33">
         <f>D6+D7</f>
         <v/>
       </c>
-      <c r="E8" s="15">
+      <c r="E8" s="33">
         <f>E6+E7</f>
         <v/>
       </c>
-      <c r="F8" s="15">
+      <c r="F8" s="33">
         <f>F6+F7</f>
         <v/>
       </c>
@@ -1664,23 +1695,23 @@
           <t>Margine EBITDA gruppo</t>
         </is>
       </c>
-      <c r="B9" s="20">
+      <c r="B9" s="36">
         <f>IFERROR(B8/B5,0)</f>
         <v/>
       </c>
-      <c r="C9" s="20">
+      <c r="C9" s="36">
         <f>IFERROR(C8/C5,0)</f>
         <v/>
       </c>
-      <c r="D9" s="20">
+      <c r="D9" s="36">
         <f>IFERROR(D8/D5,0)</f>
         <v/>
       </c>
-      <c r="E9" s="20">
+      <c r="E9" s="36">
         <f>IFERROR(E8/E5,0)</f>
         <v/>
       </c>
-      <c r="F9" s="20">
+      <c r="F9" s="36">
         <f>IFERROR(F8/F5,0)</f>
         <v/>
       </c>
@@ -1703,7 +1734,7 @@
           <t>Enterprise Value all'exit (EBITDA A5 x multiplo)</t>
         </is>
       </c>
-      <c r="B12" s="15">
+      <c r="B12" s="33">
         <f>F8*Assunzioni!B11</f>
         <v/>
       </c>
@@ -1749,19 +1780,19 @@
           <t>Investitore seed (€500k)</t>
         </is>
       </c>
-      <c r="B16" s="20">
+      <c r="B16" s="36">
         <f>Assunzioni!B29/Assunzioni!B30</f>
         <v/>
       </c>
-      <c r="C16" s="20">
+      <c r="C16" s="36">
         <f>B16*(1-Assunzioni!B31/Assunzioni!B32-Assunzioni!B33)</f>
         <v/>
       </c>
-      <c r="D16" s="13">
+      <c r="D16" s="31">
         <f>C16*B12</f>
         <v/>
       </c>
-      <c r="E16" s="16">
+      <c r="E16" s="34">
         <f>D16/Assunzioni!B29</f>
         <v/>
       </c>
@@ -1772,15 +1803,15 @@
           <t>Investitore round di scala</t>
         </is>
       </c>
-      <c r="C17" s="20">
+      <c r="C17" s="36">
         <f>Assunzioni!B31/Assunzioni!B32</f>
         <v/>
       </c>
-      <c r="D17" s="13">
+      <c r="D17" s="31">
         <f>C17*B12</f>
         <v/>
       </c>
-      <c r="E17" s="16">
+      <c r="E17" s="34">
         <f>D17/Assunzioni!B31</f>
         <v/>
       </c>
@@ -1791,11 +1822,11 @@
           <t>Pool ESOP (management + COO)</t>
         </is>
       </c>
-      <c r="C18" s="20">
+      <c r="C18" s="36">
         <f>Assunzioni!B33</f>
         <v/>
       </c>
-      <c r="D18" s="13">
+      <c r="D18" s="31">
         <f>C18*B12</f>
         <v/>
       </c>
@@ -1806,15 +1837,15 @@
           <t>Fondatori (Luca, Diana, Marcello)</t>
         </is>
       </c>
-      <c r="B19" s="20">
+      <c r="B19" s="36">
         <f>1-B16</f>
         <v/>
       </c>
-      <c r="C19" s="22">
+      <c r="C19" s="37">
         <f>1-C16-C17-C18</f>
         <v/>
       </c>
-      <c r="D19" s="15">
+      <c r="D19" s="33">
         <f>C19*B12</f>
         <v/>
       </c>
@@ -1825,7 +1856,7 @@
           <t>Totale (check = 100%)</t>
         </is>
       </c>
-      <c r="C20" s="23">
+      <c r="C20" s="38">
         <f>C16+C17+C18+C19</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Venere: seed a €700k (seed-pilota), post-money ~4,5M (~15,6% ceduto); deck e modello allineati
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QhepYozFjjk17WbLpFAXS3
</commit_message>
<xml_diff>
--- a/Venere_Modello_Finanziario.xlsx
+++ b/Venere_Modello_Finanziario.xlsx
@@ -987,11 +987,11 @@
         </is>
       </c>
       <c r="B29" s="30" t="n">
-        <v>500000</v>
+        <v>700000</v>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>provare 1 ambulatorio pilota + blindare 3 LOI</t>
+          <t>seed-pilota: 1 ambulatorio pilota completo + 3 LOI blindate</t>
         </is>
       </c>
     </row>
@@ -1002,11 +1002,11 @@
         </is>
       </c>
       <c r="B30" s="30" t="n">
-        <v>3500000</v>
+        <v>4500000</v>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>valutazione ipotizzata</t>
+          <t>post-money indicativo (~15% ceduto); floor 3,5M (20%)</t>
         </is>
       </c>
     </row>
@@ -1087,11 +1087,11 @@
         </is>
       </c>
       <c r="B37" s="26" t="n">
-        <v>295000</v>
+        <v>350000</v>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>contenuto; il capex pieno ~350k arriva in Series A</t>
+          <t>capex pieno sul pilota (con €700k te lo puoi permettere)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Venere: unit economics riviste e difendibili (grande centro 650k->1,2M, EBITDA ~100k->300k, MOIC/sede 3,4x); aggregati coerenti (gruppo A5 ~4M EBITDA, EV ~31,7M); deck con font piu grandi e meno spazio bianco; modello allineato
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QhepYozFjjk17WbLpFAXS3
</commit_message>
<xml_diff>
--- a/Venere_Modello_Finanziario.xlsx
+++ b/Venere_Modello_Finanziario.xlsx
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="B5" s="26" t="n">
-        <v>600000</v>
+        <v>650000</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
@@ -757,11 +757,11 @@
         </is>
       </c>
       <c r="B7" s="26" t="n">
-        <v>270000</v>
+        <v>350000</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>circa 3x EBITDA normalizzato (con clientela)</t>
+          <t>circa 3,5x EBITDA normalizzato (grande centro)</t>
         </is>
       </c>
     </row>
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="B9" s="26" t="n">
-        <v>1100000</v>
+        <v>1200000</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -807,11 +807,11 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>0.28</v>
+        <v>0.25</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>netto dei medici condivisi (pagati a prestazione)</t>
+          <t>medspa maturi 20-28%; prudente 25%</t>
         </is>
       </c>
     </row>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="B18" s="29" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="19">
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="B19" s="29" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="21">
@@ -1072,11 +1072,11 @@
         </is>
       </c>
       <c r="B36" s="26" t="n">
-        <v>175000</v>
+        <v>200000</v>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>circa 65% del prezzo (o pilota economico + rollover)</t>
+          <t>cash al closing pilota (con rollover del venditore)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Venere: gate del seed abbassato a 1a LOI firmata + pipeline (ambulatori: 3 LOI troppo); seed €700k coerente ovunque (deck, memo, piani, modello, PDF)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QhepYozFjjk17WbLpFAXS3
</commit_message>
<xml_diff>
--- a/Venere_Modello_Finanziario.xlsx
+++ b/Venere_Modello_Finanziario.xlsx
@@ -991,7 +991,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>seed-pilota: 1 ambulatorio pilota completo + 3 LOI blindate</t>
+          <t>seed-pilota: 1 ambulatorio pilota (gate: 1a LOI firmata + pipeline)</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1492,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Lettura onesta: €500k converte 1 ambulatorio PILOTA e blinda 3 LOI (margine sottile). La conversione piena dei 3 e' la Series A (~€1,6M). Per un pilota comodo servirebbero ~€600-700k.</t>
+          <t>Lettura onesta: €700k converte 1 ambulatorio PILOTA e apre il seed con la 1a LOI firmata + pipeline. La scala dei centri successivi e' la Series A. Con €700k il pilota ha runway comodo.</t>
         </is>
       </c>
     </row>

</xml_diff>